<commit_message>
Update the Main PCB Excel BOM
</commit_message>
<xml_diff>
--- a/Hardware/Running_Hardware/Open_STMPLC_IO_V0.1/bom/IO_PCB.xlsx
+++ b/Hardware/Running_Hardware/Open_STMPLC_IO_V0.1/bom/IO_PCB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/319af35e91399a73/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Open_PLCSTM32\Open_STMPLC\Hardware\Running_Hardware\Open_STMPLC_IO_V0.1\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="99" documentId="8_{27EE40A1-620B-40E3-84C2-492604364477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C852DD1-8F4C-49DB-B257-7058B8D6DC26}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F78FEE7E-8E37-49F4-813A-F9A663C709BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{A8173578-5B5D-445A-B535-9A2B2779D8C5}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{A8173578-5B5D-445A-B535-9A2B2779D8C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>